<commit_message>
UPdate to the schema and the melpay.xsls file
</commit_message>
<xml_diff>
--- a/Melpay.xlsx
+++ b/Melpay.xlsx
@@ -125,7 +125,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -257,7 +257,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.55"/>
@@ -295,7 +295,7 @@
       <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>701450691</v>
       </c>
     </row>
@@ -304,7 +304,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>45414</v>
@@ -312,7 +312,7 @@
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>701450692</v>
       </c>
     </row>
@@ -329,7 +329,7 @@
       <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>701450693</v>
       </c>
     </row>
@@ -338,7 +338,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>1500</v>
+        <v>5477</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>45417</v>
@@ -346,7 +346,7 @@
       <c r="D5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>701450694</v>
       </c>
     </row>
@@ -363,7 +363,7 @@
       <c r="D6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="1" t="n">
         <v>701450695</v>
       </c>
     </row>

</xml_diff>